<commit_message>
feat(registre-formulations): famille d'exclusion déclarée — 135 formulations archaïques écartées (verdict RF 2026-09-09)
registre_formulations.yaml (forme source exacte, motif, validation
datée), chargé par charge_politique, appliqué dans
_candidates_formulations avant R3. OFS/ANS refusés au chargement ;
famille LLM couverte par fixture. Témoins : paires écartée/gardée à
même sonde (tabès A52.1, croup A36.0/B94.8), fiche I64 avant/après,
hors-Formulations byte-identique, ancrage des entrées sur le CSV.
Support de relecture synchronisé sur les verdicts. 869 tests verts.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/scripts/explore/relectures/relecture_registre_formulations_v1.xlsx
+++ b/scripts/explore/relectures/relecture_registre_formulations_v1.xlsx
@@ -1,16 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/remi/Documents/recode-icd/scripts/explore/relectures/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ABA9533-99CD-4B49-B427-650C8B173599}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="500" windowWidth="48640" windowHeight="23520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="candidates" sheetId="1" r:id="rId1"/>
     <sheet name="fiches_impact" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -1385,11 +1391,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="#,##0;[Red]-#,##0"/>
+    <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1431,54 +1437,64 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
-    <dxf/>
     <dxf>
-      <numFmt numFmtId="164" formatCode="#,##0;[Red]-#,##0"/>
+      <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="#,##0;[Red]\-#,##0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:J158" totalsRowShown="0">
-  <autoFilter ref="A1:J158"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Frame0" displayName="Frame0" ref="A1:J158" totalsRowShown="0">
+  <autoFilter ref="A1:J158" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="10">
-    <tableColumn id="1" name="code" dataDxfId="0"/>
-    <tableColumn id="2" name="libelle_officiel" dataDxfId="0"/>
-    <tableColumn id="3" name="chapitre" dataDxfId="0"/>
-    <tableColumn id="4" name="forme_rendue" dataDxfId="0"/>
-    <tableColumn id="5" name="forme_source" dataDxfId="0"/>
-    <tableColumn id="6" name="source" dataDxfId="0"/>
-    <tableColumn id="7" name="signal" dataDxfId="0"/>
-    <tableColumn id="8" name="proposition" dataDxfId="0"/>
-    <tableColumn id="9" name="motif" dataDxfId="0"/>
-    <tableColumn id="10" name="version_regle" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="code"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="libelle_officiel"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="chapitre"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="forme_rendue"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="forme_source"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="source"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="signal"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="proposition"/>
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="motif"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="version_regle"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Frame1" displayName="Frame1" ref="A1:G9" totalsRowShown="0">
-  <autoFilter ref="A1:G9"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Frame1" displayName="Frame1" ref="A1:G9" totalsRowShown="0">
+  <autoFilter ref="A1:G9" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="7">
-    <tableColumn id="1" name="code" dataDxfId="0"/>
-    <tableColumn id="2" name="libelle_officiel" dataDxfId="0"/>
-    <tableColumn id="3" name="chapitre" dataDxfId="0"/>
-    <tableColumn id="4" name="formulations_avant" dataDxfId="1"/>
-    <tableColumn id="5" name="formulations_apres" dataDxfId="1"/>
-    <tableColumn id="6" name="section_videe" dataDxfId="0"/>
-    <tableColumn id="7" name="version_regle" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="code"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="libelle_officiel"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="chapitre"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="formulations_avant" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="formulations_apres" dataDxfId="0"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="section_videe"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0100-000007000000}" name="version_regle"/>
   </tableColumns>
   <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1516,7 +1532,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1550,6 +1566,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -1584,9 +1601,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1759,23 +1777,23 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J158"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="101" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.7109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="137.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="76.5703125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59" customWidth="1"/>
+    <col min="3" max="3" width="10.5" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="27.33203125" customWidth="1"/>
+    <col min="5" max="5" width="56.33203125" customWidth="1"/>
+    <col min="6" max="6" width="19.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="76.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1807,7 +1825,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -1839,7 +1857,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
@@ -1862,7 +1880,7 @@
         <v>16</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>23</v>
@@ -1871,7 +1889,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:10">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1903,7 +1921,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:10">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>26</v>
       </c>
@@ -1926,7 +1944,7 @@
         <v>30</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>31</v>
@@ -1935,7 +1953,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>26</v>
       </c>
@@ -1958,7 +1976,7 @@
         <v>30</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>31</v>
@@ -1967,7 +1985,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:10">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>26</v>
       </c>
@@ -1990,7 +2008,7 @@
         <v>30</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>31</v>
@@ -1999,7 +2017,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>35</v>
       </c>
@@ -2031,7 +2049,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>41</v>
       </c>
@@ -2054,7 +2072,7 @@
         <v>45</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I9" s="1" t="s">
         <v>46</v>
@@ -2063,7 +2081,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>41</v>
       </c>
@@ -2095,7 +2113,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>41</v>
       </c>
@@ -2127,7 +2145,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:10">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>41</v>
       </c>
@@ -2159,7 +2177,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="13" spans="1:10">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>41</v>
       </c>
@@ -2182,7 +2200,7 @@
         <v>39</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I13" s="1" t="s">
         <v>40</v>
@@ -2191,7 +2209,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="14" spans="1:10">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>41</v>
       </c>
@@ -2214,7 +2232,7 @@
         <v>45</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I14" s="1" t="s">
         <v>46</v>
@@ -2223,7 +2241,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:10">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>41</v>
       </c>
@@ -2255,7 +2273,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:10">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>41</v>
       </c>
@@ -2287,7 +2305,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:10">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>55</v>
       </c>
@@ -2319,7 +2337,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:10">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>60</v>
       </c>
@@ -2351,7 +2369,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:10">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>63</v>
       </c>
@@ -2374,7 +2392,7 @@
         <v>68</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I19" s="1" t="s">
         <v>69</v>
@@ -2383,7 +2401,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:10">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>70</v>
       </c>
@@ -2415,7 +2433,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:10">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>75</v>
       </c>
@@ -2447,7 +2465,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:10">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>81</v>
       </c>
@@ -2479,7 +2497,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:10">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>81</v>
       </c>
@@ -2511,7 +2529,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:10">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>87</v>
       </c>
@@ -2543,7 +2561,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:10">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>91</v>
       </c>
@@ -2575,7 +2593,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:10">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>91</v>
       </c>
@@ -2607,7 +2625,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="1:10">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>96</v>
       </c>
@@ -2639,7 +2657,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:10">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>96</v>
       </c>
@@ -2671,7 +2689,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="1:10">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>101</v>
       </c>
@@ -2703,7 +2721,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="30" spans="1:10">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>101</v>
       </c>
@@ -2735,7 +2753,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:10">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>108</v>
       </c>
@@ -2758,7 +2776,7 @@
         <v>112</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>18</v>
@@ -2767,7 +2785,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="1:10">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>108</v>
       </c>
@@ -2799,7 +2817,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="33" spans="1:10">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>108</v>
       </c>
@@ -2831,7 +2849,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="34" spans="1:10">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>108</v>
       </c>
@@ -2863,7 +2881,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:10">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>117</v>
       </c>
@@ -2895,7 +2913,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:10">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>117</v>
       </c>
@@ -2927,7 +2945,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="37" spans="1:10">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>117</v>
       </c>
@@ -2959,7 +2977,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:10">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>117</v>
       </c>
@@ -2991,7 +3009,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:10">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>117</v>
       </c>
@@ -3023,7 +3041,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:10">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>129</v>
       </c>
@@ -3055,7 +3073,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="41" spans="1:10">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>132</v>
       </c>
@@ -3087,7 +3105,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="42" spans="1:10">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>136</v>
       </c>
@@ -3119,7 +3137,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="43" spans="1:10">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>140</v>
       </c>
@@ -3151,7 +3169,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="44" spans="1:10">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>145</v>
       </c>
@@ -3183,7 +3201,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="45" spans="1:10">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>145</v>
       </c>
@@ -3215,7 +3233,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="46" spans="1:10">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>145</v>
       </c>
@@ -3247,7 +3265,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:10">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>145</v>
       </c>
@@ -3279,7 +3297,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:10">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>145</v>
       </c>
@@ -3311,7 +3329,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="49" spans="1:10">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>145</v>
       </c>
@@ -3343,7 +3361,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="50" spans="1:10">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>145</v>
       </c>
@@ -3375,7 +3393,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="51" spans="1:10">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>145</v>
       </c>
@@ -3407,7 +3425,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="52" spans="1:10">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>145</v>
       </c>
@@ -3439,7 +3457,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:10">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>145</v>
       </c>
@@ -3471,7 +3489,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="54" spans="1:10">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>145</v>
       </c>
@@ -3503,7 +3521,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="55" spans="1:10">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>145</v>
       </c>
@@ -3535,7 +3553,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="56" spans="1:10">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>145</v>
       </c>
@@ -3567,7 +3585,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="57" spans="1:10">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>145</v>
       </c>
@@ -3599,7 +3617,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="58" spans="1:10">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>174</v>
       </c>
@@ -3631,7 +3649,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="59" spans="1:10">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>174</v>
       </c>
@@ -3663,7 +3681,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="60" spans="1:10">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>180</v>
       </c>
@@ -3695,7 +3713,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="61" spans="1:10">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>180</v>
       </c>
@@ -3727,7 +3745,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="62" spans="1:10">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>186</v>
       </c>
@@ -3759,7 +3777,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="63" spans="1:10">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>186</v>
       </c>
@@ -3791,7 +3809,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="64" spans="1:10">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>186</v>
       </c>
@@ -3823,7 +3841,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="65" spans="1:10">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>186</v>
       </c>
@@ -3855,7 +3873,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="66" spans="1:10">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>186</v>
       </c>
@@ -3887,7 +3905,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="67" spans="1:10">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>186</v>
       </c>
@@ -3919,7 +3937,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="68" spans="1:10">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>186</v>
       </c>
@@ -3951,7 +3969,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="69" spans="1:10">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>186</v>
       </c>
@@ -3983,7 +4001,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="70" spans="1:10">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>186</v>
       </c>
@@ -4015,7 +4033,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="71" spans="1:10">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>186</v>
       </c>
@@ -4047,7 +4065,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="72" spans="1:10">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>186</v>
       </c>
@@ -4079,7 +4097,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="73" spans="1:10">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>186</v>
       </c>
@@ -4111,7 +4129,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="74" spans="1:10">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>200</v>
       </c>
@@ -4143,7 +4161,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="75" spans="1:10">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>204</v>
       </c>
@@ -4175,7 +4193,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="76" spans="1:10">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>208</v>
       </c>
@@ -4207,7 +4225,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="77" spans="1:10">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>212</v>
       </c>
@@ -4239,7 +4257,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="78" spans="1:10">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>215</v>
       </c>
@@ -4271,7 +4289,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="79" spans="1:10">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>220</v>
       </c>
@@ -4303,7 +4321,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="80" spans="1:10">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>224</v>
       </c>
@@ -4335,7 +4353,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="81" spans="1:10">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>229</v>
       </c>
@@ -4367,7 +4385,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="82" spans="1:10">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>229</v>
       </c>
@@ -4399,7 +4417,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="83" spans="1:10">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>233</v>
       </c>
@@ -4431,7 +4449,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="84" spans="1:10">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>235</v>
       </c>
@@ -4463,7 +4481,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="85" spans="1:10">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>235</v>
       </c>
@@ -4495,7 +4513,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="86" spans="1:10">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>235</v>
       </c>
@@ -4527,7 +4545,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="87" spans="1:10">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>235</v>
       </c>
@@ -4559,7 +4577,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="88" spans="1:10">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>235</v>
       </c>
@@ -4591,7 +4609,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="89" spans="1:10">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>235</v>
       </c>
@@ -4623,7 +4641,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="90" spans="1:10">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>235</v>
       </c>
@@ -4655,7 +4673,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="91" spans="1:10">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>235</v>
       </c>
@@ -4687,7 +4705,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="92" spans="1:10">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>235</v>
       </c>
@@ -4719,7 +4737,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="93" spans="1:10">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>235</v>
       </c>
@@ -4751,7 +4769,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="94" spans="1:10">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>235</v>
       </c>
@@ -4783,7 +4801,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="95" spans="1:10">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>252</v>
       </c>
@@ -4815,7 +4833,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="96" spans="1:10">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>256</v>
       </c>
@@ -4847,7 +4865,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="97" spans="1:10">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>256</v>
       </c>
@@ -4879,7 +4897,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="98" spans="1:10">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>264</v>
       </c>
@@ -4911,7 +4929,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="99" spans="1:10">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>268</v>
       </c>
@@ -4943,7 +4961,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="100" spans="1:10">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>275</v>
       </c>
@@ -4975,7 +4993,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="101" spans="1:10">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>278</v>
       </c>
@@ -5007,7 +5025,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="102" spans="1:10">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>278</v>
       </c>
@@ -5039,7 +5057,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="103" spans="1:10">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>278</v>
       </c>
@@ -5071,7 +5089,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="104" spans="1:10">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>283</v>
       </c>
@@ -5103,7 +5121,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="105" spans="1:10">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>286</v>
       </c>
@@ -5135,7 +5153,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="106" spans="1:10">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>286</v>
       </c>
@@ -5167,7 +5185,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="107" spans="1:10">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>286</v>
       </c>
@@ -5199,7 +5217,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="108" spans="1:10">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>286</v>
       </c>
@@ -5231,7 +5249,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="109" spans="1:10">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>286</v>
       </c>
@@ -5263,7 +5281,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="110" spans="1:10">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>286</v>
       </c>
@@ -5295,7 +5313,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="111" spans="1:10">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>286</v>
       </c>
@@ -5327,7 +5345,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="112" spans="1:10">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>303</v>
       </c>
@@ -5359,7 +5377,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="113" spans="1:10">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>306</v>
       </c>
@@ -5391,7 +5409,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="114" spans="1:10">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>306</v>
       </c>
@@ -5423,7 +5441,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="115" spans="1:10">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>310</v>
       </c>
@@ -5455,7 +5473,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="116" spans="1:10">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>310</v>
       </c>
@@ -5487,7 +5505,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="117" spans="1:10">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>310</v>
       </c>
@@ -5519,7 +5537,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="118" spans="1:10">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>315</v>
       </c>
@@ -5551,7 +5569,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="119" spans="1:10">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>320</v>
       </c>
@@ -5574,7 +5592,7 @@
         <v>30</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I119" s="1" t="s">
         <v>31</v>
@@ -5583,7 +5601,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="120" spans="1:10">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>320</v>
       </c>
@@ -5606,7 +5624,7 @@
         <v>30</v>
       </c>
       <c r="H120" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I120" s="1" t="s">
         <v>31</v>
@@ -5615,7 +5633,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="121" spans="1:10">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>326</v>
       </c>
@@ -5647,7 +5665,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="122" spans="1:10">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>326</v>
       </c>
@@ -5679,7 +5697,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="123" spans="1:10">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>330</v>
       </c>
@@ -5711,7 +5729,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="124" spans="1:10">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>334</v>
       </c>
@@ -5743,7 +5761,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="125" spans="1:10">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>338</v>
       </c>
@@ -5775,7 +5793,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="126" spans="1:10">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>342</v>
       </c>
@@ -5798,7 +5816,7 @@
         <v>139</v>
       </c>
       <c r="H126" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I126" s="1" t="s">
         <v>345</v>
@@ -5807,7 +5825,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="127" spans="1:10">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>346</v>
       </c>
@@ -5830,7 +5848,7 @@
         <v>139</v>
       </c>
       <c r="H127" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I127" s="1" t="s">
         <v>345</v>
@@ -5839,7 +5857,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="128" spans="1:10">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>348</v>
       </c>
@@ -5871,7 +5889,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="129" spans="1:10">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>351</v>
       </c>
@@ -5903,7 +5921,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="130" spans="1:10">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>354</v>
       </c>
@@ -5935,7 +5953,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="131" spans="1:10">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>359</v>
       </c>
@@ -5967,7 +5985,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="132" spans="1:10">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>363</v>
       </c>
@@ -5999,7 +6017,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="133" spans="1:10">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>366</v>
       </c>
@@ -6031,7 +6049,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="134" spans="1:10">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>369</v>
       </c>
@@ -6063,7 +6081,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="135" spans="1:10">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>372</v>
       </c>
@@ -6095,7 +6113,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="136" spans="1:10">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>378</v>
       </c>
@@ -6127,7 +6145,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="137" spans="1:10">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>385</v>
       </c>
@@ -6150,7 +6168,7 @@
         <v>290</v>
       </c>
       <c r="H137" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I137" s="1" t="s">
         <v>389</v>
@@ -6159,7 +6177,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="138" spans="1:10">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>390</v>
       </c>
@@ -6191,7 +6209,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="139" spans="1:10">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>396</v>
       </c>
@@ -6223,7 +6241,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="140" spans="1:10">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>399</v>
       </c>
@@ -6255,7 +6273,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="141" spans="1:10">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>404</v>
       </c>
@@ -6287,7 +6305,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="142" spans="1:10">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>408</v>
       </c>
@@ -6319,7 +6337,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="143" spans="1:10">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>408</v>
       </c>
@@ -6351,7 +6369,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="144" spans="1:10">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>412</v>
       </c>
@@ -6374,7 +6392,7 @@
         <v>68</v>
       </c>
       <c r="H144" s="1" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="I144" s="1" t="s">
         <v>69</v>
@@ -6383,7 +6401,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="145" spans="1:10">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>416</v>
       </c>
@@ -6415,7 +6433,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="146" spans="1:10">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>416</v>
       </c>
@@ -6447,7 +6465,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="147" spans="1:10">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>416</v>
       </c>
@@ -6479,7 +6497,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="148" spans="1:10">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>422</v>
       </c>
@@ -6511,7 +6529,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="149" spans="1:10">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>426</v>
       </c>
@@ -6543,7 +6561,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="150" spans="1:10">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>429</v>
       </c>
@@ -6575,7 +6593,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="151" spans="1:10">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>433</v>
       </c>
@@ -6607,7 +6625,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="152" spans="1:10">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>436</v>
       </c>
@@ -6639,7 +6657,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="153" spans="1:10">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>440</v>
       </c>
@@ -6671,7 +6689,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="154" spans="1:10">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>440</v>
       </c>
@@ -6703,7 +6721,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="155" spans="1:10">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>445</v>
       </c>
@@ -6735,7 +6753,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="156" spans="1:10">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>445</v>
       </c>
@@ -6767,7 +6785,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="157" spans="1:10">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>445</v>
       </c>
@@ -6799,7 +6817,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="158" spans="1:10">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>445</v>
       </c>
@@ -6840,19 +6858,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="76.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="20.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="7.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="76.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="20.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6875,7 +6893,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>75</v>
       </c>
@@ -6898,7 +6916,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
@@ -6921,7 +6939,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>87</v>
       </c>
@@ -6944,7 +6962,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>91</v>
       </c>
@@ -6967,7 +6985,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>174</v>
       </c>
@@ -6990,7 +7008,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>256</v>
       </c>
@@ -7013,7 +7031,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>286</v>
       </c>
@@ -7036,7 +7054,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>330</v>
       </c>

</xml_diff>